<commit_message>
thêm SRS và cập nhật tài liệu
</commit_message>
<xml_diff>
--- a/docs/Nhóm 16/01 - Tai lieu du an/2. Ke hoach du an phan mem/Quan_Ly_Rui_Ro_BlueMoon.xlsx
+++ b/docs/Nhóm 16/01 - Tai lieu du an/2. Ke hoach du an phan mem/Quan_Ly_Rui_Ro_BlueMoon.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\download\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\BlueMoon\docs\Nhóm 16\01 - Tai lieu du an\2. Ke hoach du an phan mem\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{491C3AD6-18DF-46EC-9440-1AA55F104B2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29C0D4E2-7839-4625-8F65-25242E1F78C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Danh sách rủi ro" sheetId="1" r:id="rId1"/>
@@ -102,9 +102,6 @@
     <t>Sắp xếp công việc theo thứ tự ưu tiên và phụ thuộc; theo dõi tiến độ hàng ngày; điều chỉnh Sprint Backlog trong Retrospective</t>
   </si>
   <si>
-    <t>Rủi ro kỹ thuật: nhóm chưa quen JavaFX hoặc MySQL</t>
-  </si>
-  <si>
     <t>Phân công thành viên tìm hiểu trước Sprint 0; tổ chức buổi chia sẻ kỹ thuật nội bộ; tham khảo tài liệu chính thức và ví dụ mẫu</t>
   </si>
   <si>
@@ -219,9 +216,6 @@
     <t>Chậm trễ từ Sprint trước</t>
   </si>
   <si>
-    <t>Rủi ro kỹ thuật (JavaFX, MySQL)</t>
-  </si>
-  <si>
     <t>Khách hàng từ chối nghiệm thu</t>
   </si>
   <si>
@@ -262,6 +256,12 @@
   </si>
   <si>
     <t xml:space="preserve">Nhóm 6  |  Môn: Nhập môn Công nghệ Phần mềm  |  SoICT – HUST  |  Phiên bản: v1.0 </t>
+  </si>
+  <si>
+    <t>Rủi ro kỹ thuật: nhóm chưa quen dùng SpringBoot, CSS hoặc MySQL</t>
+  </si>
+  <si>
+    <t>Rủi ro kỹ thuật</t>
   </si>
 </sst>
 </file>
@@ -808,7 +808,7 @@
     </row>
     <row r="2" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="22" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B2" s="19"/>
       <c r="C2" s="19"/>
@@ -961,7 +961,7 @@
         <v>6</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>25</v>
+        <v>77</v>
       </c>
       <c r="C10" s="5" t="s">
         <v>14</v>
@@ -973,10 +973,10 @@
         <v>15</v>
       </c>
       <c r="F10" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="G10" s="5" t="s">
         <v>26</v>
-      </c>
-      <c r="G10" s="5" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="52.05" customHeight="1" x14ac:dyDescent="0.25">
@@ -984,7 +984,7 @@
         <v>7</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>14</v>
@@ -996,7 +996,7 @@
         <v>15</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G11" s="2" t="s">
         <v>17</v>
@@ -1007,19 +1007,19 @@
         <v>8</v>
       </c>
       <c r="B12" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="F12" s="6" t="s">
         <v>30</v>
-      </c>
-      <c r="C12" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="D12" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E12" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="F12" s="6" t="s">
-        <v>31</v>
       </c>
       <c r="G12" s="5" t="s">
         <v>12</v>
@@ -1030,7 +1030,7 @@
         <v>9</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>9</v>
@@ -1042,10 +1042,10 @@
         <v>15</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="52.05" customHeight="1" x14ac:dyDescent="0.25">
@@ -1053,7 +1053,7 @@
         <v>10</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C14" s="5" t="s">
         <v>14</v>
@@ -1065,15 +1065,15 @@
         <v>10</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="21" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B16" s="19"/>
       <c r="C16" s="19"/>
@@ -1084,10 +1084,10 @@
     </row>
     <row r="17" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="B17" s="18" t="s">
         <v>37</v>
-      </c>
-      <c r="B17" s="18" t="s">
-        <v>38</v>
       </c>
       <c r="C17" s="19"/>
       <c r="D17" s="19"/>
@@ -1097,10 +1097,10 @@
     </row>
     <row r="18" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="B18" s="18" t="s">
         <v>39</v>
-      </c>
-      <c r="B18" s="18" t="s">
-        <v>40</v>
       </c>
       <c r="C18" s="19"/>
       <c r="D18" s="19"/>
@@ -1110,10 +1110,10 @@
     </row>
     <row r="19" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="B19" s="18" t="s">
         <v>41</v>
-      </c>
-      <c r="B19" s="18" t="s">
-        <v>42</v>
       </c>
       <c r="C19" s="19"/>
       <c r="D19" s="19"/>
@@ -1123,10 +1123,10 @@
     </row>
     <row r="20" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="B20" s="18" t="s">
         <v>43</v>
-      </c>
-      <c r="B20" s="18" t="s">
-        <v>44</v>
       </c>
       <c r="C20" s="19"/>
       <c r="D20" s="19"/>
@@ -1136,10 +1136,10 @@
     </row>
     <row r="21" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="B21" s="18" t="s">
         <v>45</v>
-      </c>
-      <c r="B21" s="18" t="s">
-        <v>46</v>
       </c>
       <c r="C21" s="19"/>
       <c r="D21" s="19"/>
@@ -1149,10 +1149,10 @@
     </row>
     <row r="22" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="B22" s="18" t="s">
         <v>47</v>
-      </c>
-      <c r="B22" s="18" t="s">
-        <v>48</v>
       </c>
       <c r="C22" s="19"/>
       <c r="D22" s="19"/>
@@ -1187,7 +1187,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="31.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="20" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B1" s="19"/>
       <c r="C1" s="19"/>
@@ -1196,7 +1196,7 @@
     </row>
     <row r="3" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B3" s="9" t="s">
         <v>14</v>
@@ -1213,7 +1213,7 @@
         <v>14</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C4" s="12" t="s">
         <v>15</v>
@@ -1233,7 +1233,7 @@
         <v>10</v>
       </c>
       <c r="D5" s="14" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.25">
@@ -1244,16 +1244,16 @@
         <v>10</v>
       </c>
       <c r="C6" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="D6" s="15" t="s">
         <v>52</v>
-      </c>
-      <c r="D6" s="15" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="9" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="21" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B9" s="19"/>
       <c r="C9" s="19"/>
@@ -1265,16 +1265,16 @@
         <v>1</v>
       </c>
       <c r="B10" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C10" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="D10" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="D10" s="1" t="s">
+      <c r="E10" s="1" t="s">
         <v>57</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
@@ -1282,7 +1282,7 @@
         <v>1</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>9</v>
@@ -1299,7 +1299,7 @@
         <v>2</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C12" s="5" t="s">
         <v>9</v>
@@ -1316,7 +1316,7 @@
         <v>3</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>14</v>
@@ -1333,7 +1333,7 @@
         <v>4</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C14" s="5" t="s">
         <v>9</v>
@@ -1350,7 +1350,7 @@
         <v>5</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>14</v>
@@ -1367,7 +1367,7 @@
         <v>6</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>64</v>
+        <v>78</v>
       </c>
       <c r="C16" s="5" t="s">
         <v>14</v>
@@ -1384,7 +1384,7 @@
         <v>7</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C17" s="2" t="s">
         <v>14</v>
@@ -1401,7 +1401,7 @@
         <v>8</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C18" s="5" t="s">
         <v>9</v>
@@ -1418,7 +1418,7 @@
         <v>9</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C19" s="2" t="s">
         <v>9</v>
@@ -1435,7 +1435,7 @@
         <v>10</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C20" s="5" t="s">
         <v>14</v>
@@ -1471,7 +1471,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="31.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="20" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B1" s="19"/>
       <c r="C1" s="19"/>
@@ -1481,7 +1481,7 @@
     </row>
     <row r="2" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="22" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B2" s="19"/>
       <c r="C2" s="19"/>
@@ -1494,19 +1494,19 @@
         <v>1</v>
       </c>
       <c r="B4" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="E4" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="C4" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="D4" s="1" t="s">
+      <c r="F4" s="1" t="s">
         <v>72</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>74</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="52.05" customHeight="1" x14ac:dyDescent="0.25">
@@ -1514,13 +1514,13 @@
         <v>1</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>10</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="E5" s="3" t="s">
         <v>11</v>
@@ -1534,13 +1534,13 @@
         <v>2</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C6" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="E6" s="6" t="s">
         <v>16</v>
@@ -1554,13 +1554,13 @@
         <v>3</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>10</v>
       </c>
       <c r="D7" s="16" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="E7" s="3" t="s">
         <v>20</v>
@@ -1574,13 +1574,13 @@
         <v>4</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="17" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="E8" s="6" t="s">
         <v>22</v>
@@ -1594,13 +1594,13 @@
         <v>5</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C9" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D9" s="16" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="E9" s="3" t="s">
         <v>24</v>
@@ -1614,19 +1614,19 @@
         <v>6</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>64</v>
+        <v>78</v>
       </c>
       <c r="C10" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D10" s="17" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="E10" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="F10" s="5" t="s">
         <v>26</v>
-      </c>
-      <c r="F10" s="5" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="52.05" customHeight="1" x14ac:dyDescent="0.25">
@@ -1634,16 +1634,16 @@
         <v>7</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C11" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D11" s="16" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F11" s="2" t="s">
         <v>17</v>
@@ -1654,16 +1654,16 @@
         <v>8</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>10</v>
       </c>
       <c r="D12" s="17" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F12" s="5" t="s">
         <v>12</v>
@@ -1674,19 +1674,19 @@
         <v>9</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C13" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D13" s="16" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="52.05" customHeight="1" x14ac:dyDescent="0.25">
@@ -1694,19 +1694,19 @@
         <v>10</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C14" s="4" t="s">
         <v>10</v>
       </c>
       <c r="D14" s="17" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>